<commit_message>
Spruce up UI, add settings sidebar, Excel path validation, and open file feature
</commit_message>
<xml_diff>
--- a/server/data/activityTracker.xlsx
+++ b/server/data/activityTracker.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:N8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -430,6 +430,18 @@
       <c r="J1" t="str">
         <v>todayDate</v>
       </c>
+      <c r="K1" t="str">
+        <v>prevAction</v>
+      </c>
+      <c r="L1" t="str">
+        <v>followUpCount</v>
+      </c>
+      <c r="M1" t="str">
+        <v>id</v>
+      </c>
+      <c r="N1" t="str">
+        <v>status</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -463,9 +475,273 @@
         <v>2026-06-01</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>a</v>
+      </c>
+      <c r="B3" t="str">
+        <v>a</v>
+      </c>
+      <c r="C3" t="str">
+        <v>mridul.purkayastha04@gmail.com</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v>a</v>
+      </c>
+      <c r="G3" t="str">
+        <v>assd</v>
+      </c>
+      <c r="H3" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="K3" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3" t="str">
+        <v>85ade2a2-722c-41c8-93d4-8445364dca39</v>
+      </c>
+      <c r="N3" t="str">
+        <v>completed</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>a</v>
+      </c>
+      <c r="B4" t="str">
+        <v>a</v>
+      </c>
+      <c r="C4" t="str">
+        <v>mridul.purkayastha04@gmail.com</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v>follow-up 1</v>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="K4" t="str">
+        <v>New Activity</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4" t="str">
+        <v>effd2761-3b87-4468-a0f8-6f44a1c9d928</v>
+      </c>
+      <c r="N4" t="str">
+        <v>hidden</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>a</v>
+      </c>
+      <c r="B5" t="str">
+        <v>wdadwad</v>
+      </c>
+      <c r="C5" t="str">
+        <v>mridul.purkayastha04@gmail.com</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v>awdawd</v>
+      </c>
+      <c r="G5" t="str">
+        <v>wadwad</v>
+      </c>
+      <c r="H5" t="str">
+        <v>2026-06-06</v>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="K5" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5" t="str">
+        <v>9700ef7d-f0ec-4ea1-8009-a138d233f3ca</v>
+      </c>
+      <c r="N5" t="str">
+        <v>active</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>awdw</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Mridul Purkayastha</v>
+      </c>
+      <c r="C6" t="str">
+        <v>mridul@terpmail.umd.edu</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v>sometyhing</v>
+      </c>
+      <c r="G6" t="str">
+        <v>awdawdre</v>
+      </c>
+      <c r="H6" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="K6" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6" t="str">
+        <v>b338bfbb-9949-4bee-81ee-521734d85862</v>
+      </c>
+      <c r="N6" t="str">
+        <v>completed</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>awdw</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Mridul Purkayastha</v>
+      </c>
+      <c r="C7" t="str">
+        <v>mridul@terpmail.umd.edu</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v>follow-up 1</v>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="K7" t="str">
+        <v>New Activity</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7" t="str">
+        <v>9ef5fc6e-29ff-4762-9b04-6eecf03ea3e5</v>
+      </c>
+      <c r="N7" t="str">
+        <v>active</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>awdw</v>
+      </c>
+      <c r="B8" t="str">
+        <v>a</v>
+      </c>
+      <c r="C8" t="str">
+        <v>mridul.purkayastha04@gmail.com</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
+        <v>idk</v>
+      </c>
+      <c r="G8" t="str">
+        <v>idk v2</v>
+      </c>
+      <c r="H8" t="str">
+        <v>2026-06-04</v>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="K8" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8" t="str">
+        <v>6c34d4db-412c-40ac-9967-639f69be6c82</v>
+      </c>
+      <c r="N8" t="str">
+        <v>active</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update dashboard UI and add reporting features
</commit_message>
<xml_diff>
--- a/server/data/activityTracker.xlsx
+++ b/server/data/activityTracker.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -516,7 +516,7 @@
         <v>85ade2a2-722c-41c8-93d4-8445364dca39</v>
       </c>
       <c r="N3" t="str">
-        <v>completed</v>
+        <v>hidden</v>
       </c>
     </row>
     <row r="4">
@@ -604,7 +604,7 @@
         <v>9700ef7d-f0ec-4ea1-8009-a138d233f3ca</v>
       </c>
       <c r="N5" t="str">
-        <v>active</v>
+        <v>hidden</v>
       </c>
     </row>
     <row r="6">
@@ -648,7 +648,7 @@
         <v>b338bfbb-9949-4bee-81ee-521734d85862</v>
       </c>
       <c r="N6" t="str">
-        <v>completed</v>
+        <v>hidden</v>
       </c>
     </row>
     <row r="7">
@@ -692,7 +692,7 @@
         <v>9ef5fc6e-29ff-4762-9b04-6eecf03ea3e5</v>
       </c>
       <c r="N7" t="str">
-        <v>active</v>
+        <v>hidden</v>
       </c>
     </row>
     <row r="8">
@@ -736,12 +736,100 @@
         <v>6c34d4db-412c-40ac-9967-639f69be6c82</v>
       </c>
       <c r="N8" t="str">
+        <v>hidden</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>a</v>
+      </c>
+      <c r="B9" t="str">
+        <v>a</v>
+      </c>
+      <c r="C9" t="str">
+        <v>mridul@terpmail.umd.edu</v>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v>aawdw</v>
+      </c>
+      <c r="G9" t="str">
+        <v>awdwadwad</v>
+      </c>
+      <c r="H9" t="str">
+        <v>2026-05-06</v>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="K9" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L9">
+        <v>0</v>
+      </c>
+      <c r="M9" t="str">
+        <v>50b1f12c-0cd4-4a93-84e9-6e9098907b5f</v>
+      </c>
+      <c r="N9" t="str">
+        <v>active</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>a</v>
+      </c>
+      <c r="B10" t="str">
+        <v>aasd</v>
+      </c>
+      <c r="C10" t="str">
+        <v>mridul@terpmail.umd.edu</v>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v>awdaw</v>
+      </c>
+      <c r="G10" t="str">
+        <v>awdaw</v>
+      </c>
+      <c r="H10" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="K10" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L10">
+        <v>0</v>
+      </c>
+      <c r="M10" t="str">
+        <v>62f0ee7e-6f54-4f6a-9a9d-81ac35c65075</v>
+      </c>
+      <c r="N10" t="str">
         <v>active</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Implement custom Combobox and react-datepicker widgets
</commit_message>
<xml_diff>
--- a/server/data/activityTracker.xlsx
+++ b/server/data/activityTracker.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -824,12 +824,144 @@
         <v>62f0ee7e-6f54-4f6a-9a9d-81ac35c65075</v>
       </c>
       <c r="N10" t="str">
+        <v>completed</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>aaa</v>
+      </c>
+      <c r="B11" t="str">
+        <v>wadwad</v>
+      </c>
+      <c r="C11" t="str">
+        <v>mridul.purkayastha04@gmail.com</v>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
+        <v>dwdaw</v>
+      </c>
+      <c r="G11" t="str">
+        <v>wdaw</v>
+      </c>
+      <c r="H11" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="I11" t="str">
+        <v>aWDAwd</v>
+      </c>
+      <c r="J11" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="K11" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L11">
+        <v>0</v>
+      </c>
+      <c r="M11" t="str">
+        <v>a2a6b776-55df-4101-ba2f-3dab3958c1b9</v>
+      </c>
+      <c r="N11" t="str">
+        <v>completed</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>aaa</v>
+      </c>
+      <c r="B12" t="str">
+        <v>wadwad</v>
+      </c>
+      <c r="C12" t="str">
+        <v>mridul.purkayastha04@gmail.com</v>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12" t="str">
+        <v>follow-up 1</v>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
+        <v>aWDAwd</v>
+      </c>
+      <c r="J12" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="K12" t="str">
+        <v>New Activity</v>
+      </c>
+      <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12" t="str">
+        <v>572c6612-e33e-4604-abba-ba83f427a107</v>
+      </c>
+      <c r="N12" t="str">
+        <v>active</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>a</v>
+      </c>
+      <c r="B13" t="str">
+        <v>aasd</v>
+      </c>
+      <c r="C13" t="str">
+        <v>mridul@terpmail.umd.edu</v>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
+        <v>follow-up 1</v>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="K13" t="str">
+        <v>New Activity</v>
+      </c>
+      <c r="L13">
+        <v>1</v>
+      </c>
+      <c r="M13" t="str">
+        <v>49da62df-f479-4752-976d-b32f53229a35</v>
+      </c>
+      <c r="N13" t="str">
         <v>active</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Apply sort by reminderDate and tweak Today's Actions table columns
</commit_message>
<xml_diff>
--- a/server/data/activityTracker.xlsx
+++ b/server/data/activityTracker.xlsx
@@ -1,31 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ActivityTracker\server\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56A056BD-C00C-41E4-A3B9-7EEEB9198E37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
   <sheets>
     <sheet name="Activities" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <numFmts count="1">
+    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+  </numFmts>
+  <fonts count="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -54,23 +64,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -395,80 +396,232 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="11.375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="42.25" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.75" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="35.75" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.375" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:N5"/>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>accountInput</v>
+      </c>
+      <c r="B1" t="str">
+        <v>contactName</v>
+      </c>
+      <c r="C1" t="str">
+        <v>contactEmail</v>
+      </c>
+      <c r="D1" t="str">
+        <v>linkedinUrl</v>
+      </c>
+      <c r="E1" t="str">
+        <v>roleTitle</v>
+      </c>
+      <c r="F1" t="str">
+        <v>actionTaken</v>
+      </c>
+      <c r="G1" t="str">
+        <v>nextStep</v>
+      </c>
+      <c r="H1" t="str">
+        <v>reminderDate</v>
+      </c>
+      <c r="I1" t="str">
+        <v>notes</v>
+      </c>
+      <c r="J1" t="str">
+        <v>todayDate</v>
+      </c>
+      <c r="K1" t="str">
+        <v>prevAction</v>
+      </c>
+      <c r="L1" t="str">
+        <v>followUpCount</v>
+      </c>
+      <c r="M1" t="str">
+        <v>id</v>
+      </c>
+      <c r="N1" t="str">
+        <v>status</v>
+      </c>
     </row>
-    <row r="2" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>ABC</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Person 1</v>
+      </c>
+      <c r="C2" t="str">
+        <v>person1@smth.com</v>
+      </c>
+      <c r="D2" t="str">
+        <v>https://www.linkedin.com/in/mridul-purkayastha/</v>
+      </c>
+      <c r="E2" t="str">
+        <v>CEO</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Spoke to him</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="K2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2" t="str">
+        <v>880a96ce-5cfc-4e02-8905-4c146719d921</v>
+      </c>
+      <c r="N2" t="str">
+        <v>hidden</v>
+      </c>
     </row>
-    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>ABC</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Person 1</v>
+      </c>
+      <c r="C3" t="str">
+        <v>mridul.purkayastha04@gmail.com</v>
+      </c>
+      <c r="D3" t="str">
+        <v>https://www.linkedin.com/in/mridul-purkayastha/</v>
+      </c>
+      <c r="E3" t="str">
+        <v>CEO</v>
+      </c>
+      <c r="F3" t="str">
+        <v>new smth 3</v>
+      </c>
+      <c r="G3" t="str">
+        <v>abc123</v>
+      </c>
+      <c r="H3" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="K3" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3" t="str">
+        <v>2f421488-5ebc-44f5-8a47-711dce9e7e38</v>
+      </c>
+      <c r="N3" t="str">
+        <v>hidden</v>
+      </c>
     </row>
-    <row r="4" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>ABC</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Person 1</v>
+      </c>
+      <c r="C4" t="str">
+        <v>mridul.purkayastha04@gmail.com</v>
+      </c>
+      <c r="D4" t="str">
+        <v>https://www.linkedin.com/in/mridul-purkayastha/</v>
+      </c>
+      <c r="E4" t="str">
+        <v>CEO</v>
+      </c>
+      <c r="F4" t="str">
+        <v>follow-up 1</v>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="K4" t="str">
+        <v>New Activity</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4" t="str">
+        <v>7b4b5ae7-29b7-4afa-bfa0-c693c737f089</v>
+      </c>
+      <c r="N4" t="str">
+        <v>hidden</v>
+      </c>
     </row>
-    <row r="5" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>ABC</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Person 1</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v>spoke</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="K5" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5" t="str">
+        <v>c618268e-2aac-4bc4-8dc3-12d5bc1a2d86</v>
+      </c>
+      <c r="N5" t="str">
+        <v>active</v>
+      </c>
     </row>
-    <row r="6" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-    </row>
-    <row r="7" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-    </row>
-    <row r="8" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-    </row>
-    <row r="9" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-    </row>
-    <row r="10" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-    </row>
-    <row r="11" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-    </row>
-    <row r="12" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-    </row>
-    <row r="13" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-    </row>
-    <row r="14" spans="1:2" ht="15.75" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:N5"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix timezone bug for todayDate calculation
</commit_message>
<xml_diff>
--- a/server/data/activityTracker.xlsx
+++ b/server/data/activityTracker.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -445,34 +445,34 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ABC</v>
+        <v>New account 1</v>
       </c>
       <c r="B2" t="str">
-        <v>Person 1</v>
+        <v>new person 1</v>
       </c>
       <c r="C2" t="str">
-        <v>person1@smth.com</v>
+        <v>someemail@gmail.com</v>
       </c>
       <c r="D2" t="str">
         <v>https://www.linkedin.com/in/mridul-purkayastha/</v>
       </c>
       <c r="E2" t="str">
-        <v>CEO</v>
+        <v/>
       </c>
       <c r="F2" t="str">
-        <v>Spoke to him</v>
+        <v>Reached out via Linkedin</v>
       </c>
       <c r="G2" t="str">
-        <v/>
+        <v>Follow up with new product launch</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>2026-06-05</v>
       </c>
       <c r="I2" t="str">
-        <v/>
+        <v>something person 1 did</v>
       </c>
       <c r="J2" t="str">
-        <v>2026-06-05</v>
+        <v>2026-06-06</v>
       </c>
       <c r="K2" t="str">
         <v>N/A</v>
@@ -481,42 +481,42 @@
         <v>0</v>
       </c>
       <c r="M2" t="str">
-        <v>880a96ce-5cfc-4e02-8905-4c146719d921</v>
+        <v>3aef5df5-757d-405d-8462-5b180ad56083</v>
       </c>
       <c r="N2" t="str">
-        <v>hidden</v>
+        <v>active</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ABC</v>
+        <v>New account 1</v>
       </c>
       <c r="B3" t="str">
-        <v>Person 1</v>
+        <v>new person 2</v>
       </c>
       <c r="C3" t="str">
-        <v>mridul.purkayastha04@gmail.com</v>
+        <v/>
       </c>
       <c r="D3" t="str">
-        <v>https://www.linkedin.com/in/mridul-purkayastha/</v>
+        <v/>
       </c>
       <c r="E3" t="str">
-        <v>CEO</v>
+        <v/>
       </c>
       <c r="F3" t="str">
-        <v>new smth 3</v>
+        <v>spoke to this cool guy</v>
       </c>
       <c r="G3" t="str">
-        <v>abc123</v>
+        <v>some follow up</v>
       </c>
       <c r="H3" t="str">
         <v>2026-06-05</v>
       </c>
       <c r="I3" t="str">
-        <v/>
+        <v>a</v>
       </c>
       <c r="J3" t="str">
-        <v>2026-06-05</v>
+        <v>2026-06-06</v>
       </c>
       <c r="K3" t="str">
         <v>N/A</v>
@@ -525,103 +525,15 @@
         <v>0</v>
       </c>
       <c r="M3" t="str">
-        <v>2f421488-5ebc-44f5-8a47-711dce9e7e38</v>
+        <v>10318b4e-1550-4301-8eec-b58a4d61d00a</v>
       </c>
       <c r="N3" t="str">
-        <v>hidden</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>ABC</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Person 1</v>
-      </c>
-      <c r="C4" t="str">
-        <v>mridul.purkayastha04@gmail.com</v>
-      </c>
-      <c r="D4" t="str">
-        <v>https://www.linkedin.com/in/mridul-purkayastha/</v>
-      </c>
-      <c r="E4" t="str">
-        <v>CEO</v>
-      </c>
-      <c r="F4" t="str">
-        <v>follow-up 1</v>
-      </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
-      <c r="H4" t="str">
-        <v/>
-      </c>
-      <c r="I4" t="str">
-        <v/>
-      </c>
-      <c r="J4" t="str">
-        <v>2026-06-05</v>
-      </c>
-      <c r="K4" t="str">
-        <v>New Activity</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4" t="str">
-        <v>7b4b5ae7-29b7-4afa-bfa0-c693c737f089</v>
-      </c>
-      <c r="N4" t="str">
-        <v>hidden</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>ABC</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Person 1</v>
-      </c>
-      <c r="C5" t="str">
-        <v/>
-      </c>
-      <c r="D5" t="str">
-        <v/>
-      </c>
-      <c r="E5" t="str">
-        <v/>
-      </c>
-      <c r="F5" t="str">
-        <v>spoke</v>
-      </c>
-      <c r="G5" t="str">
-        <v/>
-      </c>
-      <c r="H5" t="str">
-        <v/>
-      </c>
-      <c r="I5" t="str">
-        <v/>
-      </c>
-      <c r="J5" t="str">
-        <v>2026-06-05</v>
-      </c>
-      <c r="K5" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="L5">
-        <v>0</v>
-      </c>
-      <c r="M5" t="str">
-        <v>c618268e-2aac-4bc4-8dc3-12d5bc1a2d86</v>
-      </c>
-      <c r="N5" t="str">
         <v>active</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Implement inline edit action and wider table layouts
</commit_message>
<xml_diff>
--- a/server/data/activityTracker.xlsx
+++ b/server/data/activityTracker.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -466,13 +466,13 @@
         <v>Follow up with new product launch</v>
       </c>
       <c r="H2" t="str">
-        <v>2026-06-05</v>
+        <v>2026-06-06</v>
       </c>
       <c r="I2" t="str">
         <v>something person 1 did</v>
       </c>
       <c r="J2" t="str">
-        <v>2026-06-06</v>
+        <v>2026-06-05</v>
       </c>
       <c r="K2" t="str">
         <v>N/A</v>
@@ -504,36 +504,80 @@
         <v/>
       </c>
       <c r="F3" t="str">
-        <v>spoke to this cool guy</v>
+        <v xml:space="preserve">turns out hes okay </v>
       </c>
       <c r="G3" t="str">
         <v>some follow up</v>
       </c>
       <c r="H3" t="str">
-        <v>2026-06-05</v>
+        <v>2026-06-06</v>
       </c>
       <c r="I3" t="str">
         <v>a</v>
       </c>
       <c r="J3" t="str">
-        <v>2026-06-06</v>
+        <v>2026-06-05</v>
       </c>
       <c r="K3" t="str">
         <v>N/A</v>
       </c>
       <c r="L3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M3" t="str">
         <v>10318b4e-1550-4301-8eec-b58a4d61d00a</v>
       </c>
       <c r="N3" t="str">
+        <v>active</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>New account 2</v>
+      </c>
+      <c r="B4" t="str">
+        <v>some person</v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v>omygod new guy</v>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="K4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4" t="str">
+        <v>a44415a1-63d2-4e7c-900f-647770104224</v>
+      </c>
+      <c r="N4" t="str">
         <v>active</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix nested structural div tags
</commit_message>
<xml_diff>
--- a/server/data/activityTracker.xlsx
+++ b/server/data/activityTracker.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -548,13 +548,13 @@
         <v/>
       </c>
       <c r="F4" t="str">
-        <v>omygod new guy</v>
+        <v>smth</v>
       </c>
       <c r="G4" t="str">
         <v/>
       </c>
       <c r="H4" t="str">
-        <v/>
+        <v>2026-06-05</v>
       </c>
       <c r="I4" t="str">
         <v/>
@@ -572,12 +572,56 @@
         <v>a44415a1-63d2-4e7c-900f-647770104224</v>
       </c>
       <c r="N4" t="str">
+        <v>completed</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>New account 2</v>
+      </c>
+      <c r="B5" t="str">
+        <v>some person</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v>follow-up 1</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="K5" t="str">
+        <v>New Activity</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5" t="str">
+        <v>c2e37ded-bcfe-4286-874a-339604a986c3</v>
+      </c>
+      <c r="N5" t="str">
         <v>active</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Configure Tailwind v4 for class-based dark mode
</commit_message>
<xml_diff>
--- a/server/data/activityTracker.xlsx
+++ b/server/data/activityTracker.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -598,7 +598,7 @@
         <v/>
       </c>
       <c r="H5" t="str">
-        <v/>
+        <v>2026-06-05</v>
       </c>
       <c r="I5" t="str">
         <v/>
@@ -616,12 +616,56 @@
         <v>c2e37ded-bcfe-4286-874a-339604a986c3</v>
       </c>
       <c r="N5" t="str">
+        <v>completed</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>New account 2</v>
+      </c>
+      <c r="B6" t="str">
+        <v>some person</v>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v>oh</v>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v>2026-06-07</v>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="K6" t="str">
+        <v>follow-up 1</v>
+      </c>
+      <c r="L6">
+        <v>2</v>
+      </c>
+      <c r="M6" t="str">
+        <v>eb8cb597-c054-4f62-84a4-16f4c07d5a6c</v>
+      </c>
+      <c r="N6" t="str">
         <v>active</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Further deepen light mode contrast with slate-200 and dark outlines
</commit_message>
<xml_diff>
--- a/server/data/activityTracker.xlsx
+++ b/server/data/activityTracker.xlsx
@@ -572,7 +572,7 @@
         <v>a44415a1-63d2-4e7c-900f-647770104224</v>
       </c>
       <c r="N4" t="str">
-        <v>completed</v>
+        <v>active</v>
       </c>
     </row>
     <row r="5">
@@ -616,7 +616,7 @@
         <v>c2e37ded-bcfe-4286-874a-339604a986c3</v>
       </c>
       <c r="N5" t="str">
-        <v>completed</v>
+        <v>active</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Update View Details modal with ui-avatars and darker borders
</commit_message>
<xml_diff>
--- a/server/data/activityTracker.xlsx
+++ b/server/data/activityTracker.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -484,7 +484,7 @@
         <v>3aef5df5-757d-405d-8462-5b180ad56083</v>
       </c>
       <c r="N2" t="str">
-        <v>completed</v>
+        <v>hidden</v>
       </c>
     </row>
     <row r="3">
@@ -616,7 +616,7 @@
         <v>eb8cb597-c054-4f62-84a4-16f4c07d5a6c</v>
       </c>
       <c r="N5" t="str">
-        <v>active</v>
+        <v>completed</v>
       </c>
     </row>
     <row r="6">
@@ -704,7 +704,7 @@
         <v>44430542-4384-453f-b9bd-cb17fa3a793d</v>
       </c>
       <c r="N7" t="str">
-        <v>active</v>
+        <v>hidden</v>
       </c>
     </row>
     <row r="8">
@@ -751,9 +751,53 @@
         <v>active</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>New account 2</v>
+      </c>
+      <c r="B9" t="str">
+        <v>some person</v>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v>follow-up 3</v>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="K9" t="str">
+        <v>follow-up 2</v>
+      </c>
+      <c r="L9">
+        <v>3</v>
+      </c>
+      <c r="M9" t="str">
+        <v>88738b2c-9c5f-4ee8-905a-14f3a539d57f</v>
+      </c>
+      <c r="N9" t="str">
+        <v>active</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix UI wrapping/truncation and implement latest action logic for View feature
</commit_message>
<xml_diff>
--- a/server/data/activityTracker.xlsx
+++ b/server/data/activityTracker.xlsx
@@ -443,7 +443,7 @@
         <v>status</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
         <v>New account 1</v>
       </c>
@@ -468,8 +468,28 @@
       <c r="H2" t="str">
         <v>2026-06-05</v>
       </c>
-      <c r="I2" t="str">
-        <v>something person 1 did</v>
+      <c r="I2" t="str" xml:space="preserve">
+        <v xml:space="preserve">something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+</v>
       </c>
       <c r="J2" t="str">
         <v>2026-06-05</v>
@@ -484,7 +504,7 @@
         <v>3aef5df5-757d-405d-8462-5b180ad56083</v>
       </c>
       <c r="N2" t="str">
-        <v>hidden</v>
+        <v>active</v>
       </c>
     </row>
     <row r="3">
@@ -704,7 +724,7 @@
         <v>44430542-4384-453f-b9bd-cb17fa3a793d</v>
       </c>
       <c r="N7" t="str">
-        <v>hidden</v>
+        <v>active</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Fix Additional Notes missing box and add custom scrollbars
</commit_message>
<xml_diff>
--- a/server/data/activityTracker.xlsx
+++ b/server/data/activityTracker.xlsx
@@ -470,6 +470,194 @@
       </c>
       <c r="I2" t="str" xml:space="preserve">
         <v xml:space="preserve">something person 1 did
+a
+a
+a
+a
+a
+a
+a
+a
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
+aaaaa
+aa
+aa
+a
+something person 1 did
 aaaaa
 aa
 aa

</xml_diff>

<commit_message>
Disable page scrolling when any modal is open
</commit_message>
<xml_diff>
--- a/server/data/activityTracker.xlsx
+++ b/server/data/activityTracker.xlsx
@@ -459,8 +459,15 @@
       <c r="E2" t="str">
         <v/>
       </c>
-      <c r="F2" t="str">
-        <v>Reached out via Linkedinnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnn</v>
+      <c r="F2" t="str" xml:space="preserve">
+        <v xml:space="preserve">Reached out via Linkedinnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnn
+a
+a
+a
+a
+a
+a
+a</v>
       </c>
       <c r="G2" t="str">
         <v>Follow up with new product launch</v>
@@ -468,216 +475,8 @@
       <c r="H2" t="str">
         <v>2026-06-05</v>
       </c>
-      <c r="I2" t="str" xml:space="preserve">
-        <v xml:space="preserve">something person 1 did
-a
-a
-a
-a
-a
-a
-a
-a
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-something person 1 did
-aaaaa
-aa
-aa
-a
-</v>
+      <c r="I2" t="str">
+        <v/>
       </c>
       <c r="J2" t="str">
         <v>2026-06-05</v>
@@ -827,7 +626,7 @@
         <v>completed</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" xml:space="preserve">
       <c r="A6" t="str">
         <v>New account 1</v>
       </c>
@@ -843,8 +642,23 @@
       <c r="E6" t="str">
         <v/>
       </c>
-      <c r="F6" t="str">
-        <v>follow-up 1</v>
+      <c r="F6" t="str" xml:space="preserve">
+        <v xml:space="preserve">a
+a
+a
+a
+a
+a
+a
+a
+a
+a
+a
+a
+a
+a
+a
+</v>
       </c>
       <c r="G6" t="str">
         <v/>
@@ -852,8 +666,23 @@
       <c r="H6" t="str">
         <v/>
       </c>
-      <c r="I6" t="str">
-        <v>something person 1 did</v>
+      <c r="I6" t="str" xml:space="preserve">
+        <v xml:space="preserve">a
+a
+a
+a
+a
+a
+a
+a
+aa
+a
+a
+a
+a
+a
+a
+a</v>
       </c>
       <c r="J6" t="str">
         <v>2026-06-05</v>

</xml_diff>

<commit_message>
Sales activity tracker MVP
</commit_message>
<xml_diff>
--- a/server/data/activityTracker.xlsx
+++ b/server/data/activityTracker.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -443,37 +443,30 @@
         <v>status</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
-        <v>New account 1</v>
+        <v>a</v>
       </c>
       <c r="B2" t="str">
-        <v>new person 1</v>
+        <v>a</v>
       </c>
       <c r="C2" t="str">
-        <v>someemail@gmail.com</v>
+        <v/>
       </c>
       <c r="D2" t="str">
-        <v>https://www.linkedin.com/in/mridul-purkayastha/</v>
+        <v/>
       </c>
       <c r="E2" t="str">
         <v/>
       </c>
-      <c r="F2" t="str" xml:space="preserve">
-        <v xml:space="preserve">Reached out via Linkedinnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnnn
-a
-a
-a
-a
-a
-a
-a</v>
+      <c r="F2" t="str">
+        <v>a</v>
       </c>
       <c r="G2" t="str">
-        <v>Follow up with new product launch</v>
+        <v/>
       </c>
       <c r="H2" t="str">
-        <v>2026-06-05</v>
+        <v/>
       </c>
       <c r="I2" t="str">
         <v/>
@@ -488,353 +481,15 @@
         <v>0</v>
       </c>
       <c r="M2" t="str">
-        <v>3aef5df5-757d-405d-8462-5b180ad56083</v>
+        <v>72163df1-3ad5-4c08-ba81-d042c3c187ac</v>
       </c>
       <c r="N2" t="str">
-        <v>active</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>New account 1</v>
-      </c>
-      <c r="B3" t="str">
-        <v>new person 2</v>
-      </c>
-      <c r="C3" t="str">
-        <v/>
-      </c>
-      <c r="D3" t="str">
-        <v/>
-      </c>
-      <c r="E3" t="str">
-        <v/>
-      </c>
-      <c r="F3" t="str">
-        <v xml:space="preserve">turns out hes okay </v>
-      </c>
-      <c r="G3" t="str">
-        <v>some follow up</v>
-      </c>
-      <c r="H3" t="str">
-        <v>2026-06-06</v>
-      </c>
-      <c r="I3" t="str">
-        <v>a</v>
-      </c>
-      <c r="J3" t="str">
-        <v>2026-06-05</v>
-      </c>
-      <c r="K3" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="L3">
-        <v>1</v>
-      </c>
-      <c r="M3" t="str">
-        <v>10318b4e-1550-4301-8eec-b58a4d61d00a</v>
-      </c>
-      <c r="N3" t="str">
-        <v>active</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>New account 2</v>
-      </c>
-      <c r="B4" t="str">
-        <v>some person</v>
-      </c>
-      <c r="C4" t="str">
-        <v/>
-      </c>
-      <c r="D4" t="str">
-        <v/>
-      </c>
-      <c r="E4" t="str">
-        <v/>
-      </c>
-      <c r="F4" t="str">
-        <v>abc</v>
-      </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
-      <c r="H4" t="str">
-        <v>2026-06-05</v>
-      </c>
-      <c r="I4" t="str">
-        <v/>
-      </c>
-      <c r="J4" t="str">
-        <v>2026-06-05</v>
-      </c>
-      <c r="K4" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="L4">
-        <v>0</v>
-      </c>
-      <c r="M4" t="str">
-        <v>a44415a1-63d2-4e7c-900f-647770104224</v>
-      </c>
-      <c r="N4" t="str">
-        <v>completed</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>New account 2</v>
-      </c>
-      <c r="B5" t="str">
-        <v>some person</v>
-      </c>
-      <c r="C5" t="str">
-        <v/>
-      </c>
-      <c r="D5" t="str">
-        <v/>
-      </c>
-      <c r="E5" t="str">
-        <v/>
-      </c>
-      <c r="F5" t="str">
-        <v>oh</v>
-      </c>
-      <c r="G5" t="str">
-        <v>try smth new</v>
-      </c>
-      <c r="H5" t="str">
-        <v>2026-06-05</v>
-      </c>
-      <c r="I5" t="str">
-        <v/>
-      </c>
-      <c r="J5" t="str">
-        <v>2026-06-05</v>
-      </c>
-      <c r="K5" t="str">
-        <v>follow-up 1</v>
-      </c>
-      <c r="L5">
-        <v>2</v>
-      </c>
-      <c r="M5" t="str">
-        <v>eb8cb597-c054-4f62-84a4-16f4c07d5a6c</v>
-      </c>
-      <c r="N5" t="str">
-        <v>completed</v>
-      </c>
-    </row>
-    <row r="6" xml:space="preserve">
-      <c r="A6" t="str">
-        <v>New account 1</v>
-      </c>
-      <c r="B6" t="str">
-        <v>new person 1</v>
-      </c>
-      <c r="C6" t="str">
-        <v>someemail@gmail.com</v>
-      </c>
-      <c r="D6" t="str">
-        <v>https://www.linkedin.com/in/mridul-purkayastha/</v>
-      </c>
-      <c r="E6" t="str">
-        <v/>
-      </c>
-      <c r="F6" t="str" xml:space="preserve">
-        <v xml:space="preserve">a
-a
-a
-a
-a
-a
-a
-a
-a
-a
-a
-a
-a
-a
-a
-</v>
-      </c>
-      <c r="G6" t="str">
-        <v/>
-      </c>
-      <c r="H6" t="str">
-        <v/>
-      </c>
-      <c r="I6" t="str" xml:space="preserve">
-        <v xml:space="preserve">a
-a
-a
-a
-a
-a
-a
-a
-aa
-a
-a
-a
-a
-a
-a
-a</v>
-      </c>
-      <c r="J6" t="str">
-        <v>2026-06-05</v>
-      </c>
-      <c r="K6" t="str">
-        <v>New Activity</v>
-      </c>
-      <c r="L6">
-        <v>1</v>
-      </c>
-      <c r="M6" t="str">
-        <v>d6f9ec8f-d408-4d55-99f3-097e4ba843bd</v>
-      </c>
-      <c r="N6" t="str">
-        <v>active</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>New account 2</v>
-      </c>
-      <c r="B7" t="str">
-        <v>some person</v>
-      </c>
-      <c r="C7" t="str">
-        <v/>
-      </c>
-      <c r="D7" t="str">
-        <v/>
-      </c>
-      <c r="E7" t="str">
-        <v/>
-      </c>
-      <c r="F7" t="str">
-        <v>aaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaa</v>
-      </c>
-      <c r="G7" t="str">
-        <v/>
-      </c>
-      <c r="H7" t="str">
-        <v/>
-      </c>
-      <c r="I7" t="str">
-        <v/>
-      </c>
-      <c r="J7" t="str">
-        <v>2026-06-05</v>
-      </c>
-      <c r="K7" t="str">
-        <v>New Activity</v>
-      </c>
-      <c r="L7">
-        <v>1</v>
-      </c>
-      <c r="M7" t="str">
-        <v>44430542-4384-453f-b9bd-cb17fa3a793d</v>
-      </c>
-      <c r="N7" t="str">
-        <v>active</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>New account 1</v>
-      </c>
-      <c r="B8" t="str">
-        <v>new person 3</v>
-      </c>
-      <c r="C8" t="str">
-        <v/>
-      </c>
-      <c r="D8" t="str">
-        <v/>
-      </c>
-      <c r="E8" t="str">
-        <v/>
-      </c>
-      <c r="F8" t="str">
-        <v>oh</v>
-      </c>
-      <c r="G8" t="str">
-        <v>weeee</v>
-      </c>
-      <c r="H8" t="str">
-        <v>2026-06-02</v>
-      </c>
-      <c r="I8" t="str">
-        <v/>
-      </c>
-      <c r="J8" t="str">
-        <v>2026-06-05</v>
-      </c>
-      <c r="K8" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="L8">
-        <v>0</v>
-      </c>
-      <c r="M8" t="str">
-        <v>65b7b519-f4df-4bd6-99fd-4f89ab7228a8</v>
-      </c>
-      <c r="N8" t="str">
-        <v>active</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>New account 2</v>
-      </c>
-      <c r="B9" t="str">
-        <v>some person</v>
-      </c>
-      <c r="C9" t="str">
-        <v/>
-      </c>
-      <c r="D9" t="str">
-        <v/>
-      </c>
-      <c r="E9" t="str">
-        <v/>
-      </c>
-      <c r="F9" t="str">
-        <v>follow-up 3</v>
-      </c>
-      <c r="G9" t="str">
-        <v/>
-      </c>
-      <c r="H9" t="str">
-        <v/>
-      </c>
-      <c r="I9" t="str">
-        <v/>
-      </c>
-      <c r="J9" t="str">
-        <v>2026-06-05</v>
-      </c>
-      <c r="K9" t="str">
-        <v>follow-up 2</v>
-      </c>
-      <c r="L9">
-        <v>3</v>
-      </c>
-      <c r="M9" t="str">
-        <v>88738b2c-9c5f-4ee8-905a-14f3a539d57f</v>
-      </c>
-      <c r="N9" t="str">
         <v>active</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>